<commit_message>
Final organized files, including full references in data spreadsheets, for publication
</commit_message>
<xml_diff>
--- a/figures/Figure2/data/computed/H2O_basalt_exps_df.xlsx
+++ b/figures/Figure2/data/computed/H2O_basalt_exps_df.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="73">
   <si>
     <t>SiO2</t>
   </si>
@@ -50,9 +50,6 @@
   </si>
   <si>
     <t>Citation</t>
-  </si>
-  <si>
-    <t>Reference Number</t>
   </si>
   <si>
     <t>Simplified Rock Type</t>
@@ -593,10 +590,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R48"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:17">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -645,13 +642,10 @@
       <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:17">
+      <c r="A2" s="1" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18">
-      <c r="A2" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="B2">
         <v>49.4</v>
@@ -687,27 +681,24 @@
         <v>0.98</v>
       </c>
       <c r="M2" t="s">
-        <v>64</v>
-      </c>
-      <c r="N2">
-        <v>6</v>
-      </c>
-      <c r="O2" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N2" t="s">
+        <v>72</v>
+      </c>
+      <c r="O2">
+        <v>1200</v>
       </c>
       <c r="P2">
-        <v>1200</v>
+        <v>163</v>
       </c>
       <c r="Q2">
-        <v>163</v>
-      </c>
-      <c r="R2">
         <v>3.324647774242676</v>
       </c>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:17">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <v>50.8</v>
@@ -743,27 +734,24 @@
         <v>1.43</v>
       </c>
       <c r="M3" t="s">
-        <v>65</v>
-      </c>
-      <c r="N3">
-        <v>8</v>
-      </c>
-      <c r="O3" t="s">
-        <v>73</v>
+        <v>64</v>
+      </c>
+      <c r="N3" t="s">
+        <v>72</v>
+      </c>
+      <c r="O3">
+        <v>1200</v>
       </c>
       <c r="P3">
-        <v>1200</v>
+        <v>201</v>
       </c>
       <c r="Q3">
-        <v>201</v>
-      </c>
-      <c r="R3">
         <v>4.738555909424233</v>
       </c>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:17">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4">
         <v>50.8</v>
@@ -799,27 +787,24 @@
         <v>1.28</v>
       </c>
       <c r="M4" t="s">
-        <v>65</v>
-      </c>
-      <c r="N4">
-        <v>8</v>
-      </c>
-      <c r="O4" t="s">
-        <v>73</v>
+        <v>64</v>
+      </c>
+      <c r="N4" t="s">
+        <v>72</v>
+      </c>
+      <c r="O4">
+        <v>1200</v>
       </c>
       <c r="P4">
-        <v>1200</v>
+        <v>206</v>
       </c>
       <c r="Q4">
-        <v>206</v>
-      </c>
-      <c r="R4">
         <v>4.262692358855726</v>
       </c>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:17">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5">
         <v>49.4</v>
@@ -855,27 +840,24 @@
         <v>1.53</v>
       </c>
       <c r="M5" t="s">
-        <v>64</v>
-      </c>
-      <c r="N5">
-        <v>6</v>
-      </c>
-      <c r="O5" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N5" t="s">
+        <v>72</v>
+      </c>
+      <c r="O5">
+        <v>1200</v>
       </c>
       <c r="P5">
-        <v>1200</v>
+        <v>232</v>
       </c>
       <c r="Q5">
-        <v>232</v>
-      </c>
-      <c r="R5">
         <v>5.095446918551387</v>
       </c>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:17">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6">
         <v>46.7</v>
@@ -911,27 +893,24 @@
         <v>1.3</v>
       </c>
       <c r="M6" t="s">
-        <v>66</v>
-      </c>
-      <c r="N6">
-        <v>7</v>
-      </c>
-      <c r="O6" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N6" t="s">
+        <v>72</v>
+      </c>
+      <c r="O6">
+        <v>1092</v>
       </c>
       <c r="P6">
-        <v>1092</v>
+        <v>270</v>
       </c>
       <c r="Q6">
-        <v>270</v>
-      </c>
-      <c r="R6">
         <v>4.485391237974454</v>
       </c>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:17">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>47.91</v>
@@ -967,27 +946,24 @@
         <v>1.6</v>
       </c>
       <c r="M7" t="s">
-        <v>66</v>
-      </c>
-      <c r="N7">
-        <v>7</v>
-      </c>
-      <c r="O7" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N7" t="s">
+        <v>72</v>
+      </c>
+      <c r="O7">
+        <v>1100</v>
       </c>
       <c r="P7">
-        <v>1100</v>
+        <v>270</v>
       </c>
       <c r="Q7">
-        <v>270</v>
-      </c>
-      <c r="R7">
         <v>5.40868334149798</v>
       </c>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:17">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8">
         <v>50.8</v>
@@ -1023,27 +999,24 @@
         <v>1.74</v>
       </c>
       <c r="M8" t="s">
-        <v>65</v>
-      </c>
-      <c r="N8">
-        <v>8</v>
-      </c>
-      <c r="O8" t="s">
-        <v>73</v>
+        <v>64</v>
+      </c>
+      <c r="N8" t="s">
+        <v>72</v>
+      </c>
+      <c r="O8">
+        <v>1200</v>
       </c>
       <c r="P8">
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="Q8">
-        <v>300</v>
-      </c>
-      <c r="R8">
         <v>5.707169014041747</v>
       </c>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:17">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9">
         <v>50.8</v>
@@ -1079,27 +1052,24 @@
         <v>1.71</v>
       </c>
       <c r="M9" t="s">
-        <v>65</v>
-      </c>
-      <c r="N9">
-        <v>8</v>
-      </c>
-      <c r="O9" t="s">
-        <v>73</v>
+        <v>64</v>
+      </c>
+      <c r="N9" t="s">
+        <v>72</v>
+      </c>
+      <c r="O9">
+        <v>1200</v>
       </c>
       <c r="P9">
-        <v>1200</v>
+        <v>310</v>
       </c>
       <c r="Q9">
-        <v>310</v>
-      </c>
-      <c r="R9">
         <v>5.614293983568396</v>
       </c>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:17">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10">
         <v>48.28</v>
@@ -1135,27 +1105,24 @@
         <v>2.2</v>
       </c>
       <c r="M10" t="s">
-        <v>66</v>
-      </c>
-      <c r="N10">
-        <v>7</v>
-      </c>
-      <c r="O10" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N10" t="s">
+        <v>72</v>
+      </c>
+      <c r="O10">
+        <v>1085</v>
       </c>
       <c r="P10">
-        <v>1085</v>
+        <v>400</v>
       </c>
       <c r="Q10">
-        <v>400</v>
-      </c>
-      <c r="R10">
         <v>7.38073197367711</v>
       </c>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:17">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11">
         <v>50.17</v>
@@ -1191,27 +1158,24 @@
         <v>1.67</v>
       </c>
       <c r="M11" t="s">
-        <v>67</v>
-      </c>
-      <c r="N11">
-        <v>22</v>
-      </c>
-      <c r="O11" t="s">
-        <v>73</v>
+        <v>66</v>
+      </c>
+      <c r="N11" t="s">
+        <v>72</v>
+      </c>
+      <c r="O11">
+        <v>1250</v>
       </c>
       <c r="P11">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="Q11">
-        <v>500</v>
-      </c>
-      <c r="R11">
         <v>5.553011717743536</v>
       </c>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:17">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12">
         <v>49.64</v>
@@ -1247,27 +1211,24 @@
         <v>2.2</v>
       </c>
       <c r="M12" t="s">
-        <v>68</v>
-      </c>
-      <c r="N12">
-        <v>5</v>
-      </c>
-      <c r="O12" t="s">
-        <v>73</v>
+        <v>67</v>
+      </c>
+      <c r="N12" t="s">
+        <v>72</v>
+      </c>
+      <c r="O12">
+        <v>1200</v>
       </c>
       <c r="P12">
-        <v>1200</v>
+        <v>505</v>
       </c>
       <c r="Q12">
-        <v>505</v>
-      </c>
-      <c r="R12">
         <v>7.011584409183143</v>
       </c>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:17">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B13">
         <v>49.7</v>
@@ -1303,27 +1264,24 @@
         <v>2.23</v>
       </c>
       <c r="M13" t="s">
-        <v>65</v>
-      </c>
-      <c r="N13">
-        <v>8</v>
-      </c>
-      <c r="O13" t="s">
-        <v>73</v>
+        <v>64</v>
+      </c>
+      <c r="N13" t="s">
+        <v>72</v>
+      </c>
+      <c r="O13">
+        <v>1200</v>
       </c>
       <c r="P13">
-        <v>1200</v>
+        <v>507</v>
       </c>
       <c r="Q13">
-        <v>507</v>
-      </c>
-      <c r="R13">
         <v>7.202396568721466</v>
       </c>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:17">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14">
         <v>49.4</v>
@@ -1359,27 +1317,24 @@
         <v>2.21</v>
       </c>
       <c r="M14" t="s">
-        <v>64</v>
-      </c>
-      <c r="N14">
-        <v>6</v>
-      </c>
-      <c r="O14" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N14" t="s">
+        <v>72</v>
+      </c>
+      <c r="O14">
+        <v>1200</v>
       </c>
       <c r="P14">
-        <v>1200</v>
+        <v>524</v>
       </c>
       <c r="Q14">
-        <v>524</v>
-      </c>
-      <c r="R14">
         <v>7.197101336452757</v>
       </c>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:17">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B15">
         <v>49.64</v>
@@ -1415,27 +1370,24 @@
         <v>2.23</v>
       </c>
       <c r="M15" t="s">
-        <v>68</v>
-      </c>
-      <c r="N15">
-        <v>5</v>
-      </c>
-      <c r="O15" t="s">
-        <v>73</v>
+        <v>67</v>
+      </c>
+      <c r="N15" t="s">
+        <v>72</v>
+      </c>
+      <c r="O15">
+        <v>1200</v>
       </c>
       <c r="P15">
-        <v>1200</v>
+        <v>532</v>
       </c>
       <c r="Q15">
-        <v>532</v>
-      </c>
-      <c r="R15">
         <v>7.100408045169955</v>
       </c>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:17">
       <c r="A16" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16">
         <v>47.98</v>
@@ -1471,27 +1423,24 @@
         <v>2.5</v>
       </c>
       <c r="M16" t="s">
-        <v>66</v>
-      </c>
-      <c r="N16">
-        <v>7</v>
-      </c>
-      <c r="O16" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N16" t="s">
+        <v>72</v>
+      </c>
+      <c r="O16">
+        <v>1120</v>
       </c>
       <c r="P16">
-        <v>1120</v>
+        <v>695</v>
       </c>
       <c r="Q16">
-        <v>695</v>
-      </c>
-      <c r="R16">
         <v>8.140145859387921</v>
       </c>
     </row>
-    <row r="17" spans="1:18">
+    <row r="17" spans="1:17">
       <c r="A17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17">
         <v>47.47</v>
@@ -1527,27 +1476,24 @@
         <v>2.6</v>
       </c>
       <c r="M17" t="s">
-        <v>66</v>
-      </c>
-      <c r="N17">
-        <v>7</v>
-      </c>
-      <c r="O17" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N17" t="s">
+        <v>72</v>
+      </c>
+      <c r="O17">
+        <v>1135</v>
       </c>
       <c r="P17">
-        <v>1135</v>
+        <v>710</v>
       </c>
       <c r="Q17">
-        <v>710</v>
-      </c>
-      <c r="R17">
         <v>8.474467787065301</v>
       </c>
     </row>
-    <row r="18" spans="1:18">
+    <row r="18" spans="1:17">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18">
         <v>50.8</v>
@@ -1583,27 +1529,24 @@
         <v>2.49</v>
       </c>
       <c r="M18" t="s">
-        <v>65</v>
-      </c>
-      <c r="N18">
-        <v>8</v>
-      </c>
-      <c r="O18" t="s">
-        <v>73</v>
+        <v>64</v>
+      </c>
+      <c r="N18" t="s">
+        <v>72</v>
+      </c>
+      <c r="O18">
+        <v>1200</v>
       </c>
       <c r="P18">
-        <v>1200</v>
+        <v>717</v>
       </c>
       <c r="Q18">
-        <v>717</v>
-      </c>
-      <c r="R18">
         <v>7.971068439042039</v>
       </c>
     </row>
-    <row r="19" spans="1:18">
+    <row r="19" spans="1:17">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19">
         <v>47.16</v>
@@ -1639,27 +1582,24 @@
         <v>3.1</v>
       </c>
       <c r="M19" t="s">
-        <v>66</v>
-      </c>
-      <c r="N19">
-        <v>7</v>
-      </c>
-      <c r="O19" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N19" t="s">
+        <v>72</v>
+      </c>
+      <c r="O19">
+        <v>1095</v>
       </c>
       <c r="P19">
-        <v>1095</v>
+        <v>800</v>
       </c>
       <c r="Q19">
-        <v>800</v>
-      </c>
-      <c r="R19">
         <v>10.09138766172143</v>
       </c>
     </row>
-    <row r="20" spans="1:18">
+    <row r="20" spans="1:17">
       <c r="A20" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20">
         <v>47.64</v>
@@ -1695,27 +1635,24 @@
         <v>2.8</v>
       </c>
       <c r="M20" t="s">
-        <v>66</v>
-      </c>
-      <c r="N20">
-        <v>7</v>
-      </c>
-      <c r="O20" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N20" t="s">
+        <v>72</v>
+      </c>
+      <c r="O20">
+        <v>1062</v>
       </c>
       <c r="P20">
-        <v>1062</v>
+        <v>800</v>
       </c>
       <c r="Q20">
-        <v>800</v>
-      </c>
-      <c r="R20">
         <v>9.33422331779817</v>
       </c>
     </row>
-    <row r="21" spans="1:18">
+    <row r="21" spans="1:17">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21">
         <v>47.65</v>
@@ -1751,27 +1688,24 @@
         <v>3.1</v>
       </c>
       <c r="M21" t="s">
-        <v>66</v>
-      </c>
-      <c r="N21">
-        <v>7</v>
-      </c>
-      <c r="O21" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N21" t="s">
+        <v>72</v>
+      </c>
+      <c r="O21">
+        <v>1045</v>
       </c>
       <c r="P21">
-        <v>1045</v>
+        <v>800</v>
       </c>
       <c r="Q21">
-        <v>800</v>
-      </c>
-      <c r="R21">
         <v>10.31724542880882</v>
       </c>
     </row>
-    <row r="22" spans="1:18">
+    <row r="22" spans="1:17">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22">
         <v>47.73</v>
@@ -1807,27 +1741,24 @@
         <v>2.5</v>
       </c>
       <c r="M22" t="s">
-        <v>66</v>
-      </c>
-      <c r="N22">
-        <v>7</v>
-      </c>
-      <c r="O22" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N22" t="s">
+        <v>72</v>
+      </c>
+      <c r="O22">
+        <v>1110</v>
       </c>
       <c r="P22">
-        <v>1110</v>
+        <v>800</v>
       </c>
       <c r="Q22">
-        <v>800</v>
-      </c>
-      <c r="R22">
         <v>8.194666874978626</v>
       </c>
     </row>
-    <row r="23" spans="1:18">
+    <row r="23" spans="1:17">
       <c r="A23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B23">
         <v>47.82</v>
@@ -1863,27 +1794,24 @@
         <v>3.1</v>
       </c>
       <c r="M23" t="s">
-        <v>66</v>
-      </c>
-      <c r="N23">
-        <v>7</v>
-      </c>
-      <c r="O23" t="s">
-        <v>73</v>
+        <v>65</v>
+      </c>
+      <c r="N23" t="s">
+        <v>72</v>
+      </c>
+      <c r="O23">
+        <v>1090</v>
       </c>
       <c r="P23">
-        <v>1090</v>
+        <v>800</v>
       </c>
       <c r="Q23">
-        <v>800</v>
-      </c>
-      <c r="R23">
         <v>10.04959350430379</v>
       </c>
     </row>
-    <row r="24" spans="1:18">
+    <row r="24" spans="1:17">
       <c r="A24" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B24">
         <v>50.17</v>
@@ -1919,27 +1847,24 @@
         <v>2.97</v>
       </c>
       <c r="M24" t="s">
-        <v>67</v>
-      </c>
-      <c r="N24">
-        <v>22</v>
-      </c>
-      <c r="O24" t="s">
-        <v>73</v>
+        <v>66</v>
+      </c>
+      <c r="N24" t="s">
+        <v>72</v>
+      </c>
+      <c r="O24">
+        <v>1250</v>
       </c>
       <c r="P24">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="Q24">
-        <v>1000</v>
-      </c>
-      <c r="R24">
         <v>9.466506423619411</v>
       </c>
     </row>
-    <row r="25" spans="1:18">
+    <row r="25" spans="1:17">
       <c r="A25" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B25">
         <v>50.17</v>
@@ -1975,27 +1900,24 @@
         <v>3.310677045931118</v>
       </c>
       <c r="M25" t="s">
-        <v>67</v>
-      </c>
-      <c r="N25">
-        <v>22</v>
-      </c>
-      <c r="O25" t="s">
-        <v>73</v>
+        <v>66</v>
+      </c>
+      <c r="N25" t="s">
+        <v>72</v>
+      </c>
+      <c r="O25">
+        <v>1250</v>
       </c>
       <c r="P25">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="Q25">
-        <v>1000</v>
-      </c>
-      <c r="R25">
         <v>10.43901849723569</v>
       </c>
     </row>
-    <row r="26" spans="1:18">
+    <row r="26" spans="1:17">
       <c r="A26" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26">
         <v>49.4</v>
@@ -2031,27 +1953,24 @@
         <v>3.14</v>
       </c>
       <c r="M26" t="s">
-        <v>64</v>
-      </c>
-      <c r="N26">
-        <v>6</v>
-      </c>
-      <c r="O26" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N26" t="s">
+        <v>72</v>
+      </c>
+      <c r="O26">
+        <v>1200</v>
       </c>
       <c r="P26">
-        <v>1200</v>
+        <v>1013</v>
       </c>
       <c r="Q26">
-        <v>1013</v>
-      </c>
-      <c r="R26">
         <v>9.925148335654777</v>
       </c>
     </row>
-    <row r="27" spans="1:18">
+    <row r="27" spans="1:17">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B27">
         <v>49.64</v>
@@ -2087,27 +2006,24 @@
         <v>3.05</v>
       </c>
       <c r="M27" t="s">
-        <v>69</v>
-      </c>
-      <c r="N27">
-        <v>5</v>
-      </c>
-      <c r="O27" t="s">
-        <v>73</v>
+        <v>68</v>
+      </c>
+      <c r="N27" t="s">
+        <v>72</v>
+      </c>
+      <c r="O27">
+        <v>1200</v>
       </c>
       <c r="P27">
-        <v>1200</v>
+        <v>1019</v>
       </c>
       <c r="Q27">
-        <v>1019</v>
-      </c>
-      <c r="R27">
         <v>9.464217982001379</v>
       </c>
     </row>
-    <row r="28" spans="1:18">
+    <row r="28" spans="1:17">
       <c r="A28" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B28">
         <v>49.64</v>
@@ -2143,27 +2059,24 @@
         <v>3.32</v>
       </c>
       <c r="M28" t="s">
-        <v>68</v>
-      </c>
-      <c r="N28">
-        <v>5</v>
-      </c>
-      <c r="O28" t="s">
-        <v>73</v>
+        <v>67</v>
+      </c>
+      <c r="N28" t="s">
+        <v>72</v>
+      </c>
+      <c r="O28">
+        <v>1200</v>
       </c>
       <c r="P28">
-        <v>1200</v>
+        <v>1023</v>
       </c>
       <c r="Q28">
-        <v>1023</v>
-      </c>
-      <c r="R28">
         <v>10.21643903734803</v>
       </c>
     </row>
-    <row r="29" spans="1:18">
+    <row r="29" spans="1:17">
       <c r="A29" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B29">
         <v>50.71</v>
@@ -2199,27 +2112,24 @@
         <v>3.09</v>
       </c>
       <c r="M29" t="s">
-        <v>70</v>
-      </c>
-      <c r="N29">
-        <v>2</v>
-      </c>
-      <c r="O29" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="N29" t="s">
+        <v>72</v>
+      </c>
+      <c r="O29">
+        <v>1100</v>
       </c>
       <c r="P29">
-        <v>1100</v>
+        <v>1034</v>
       </c>
       <c r="Q29">
-        <v>1034</v>
-      </c>
-      <c r="R29">
         <v>10.1787197799897</v>
       </c>
     </row>
-    <row r="30" spans="1:18">
+    <row r="30" spans="1:17">
       <c r="A30" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B30">
         <v>50.71</v>
@@ -2255,27 +2165,24 @@
         <v>4.59</v>
       </c>
       <c r="M30" t="s">
-        <v>70</v>
-      </c>
-      <c r="N30">
-        <v>2</v>
-      </c>
-      <c r="O30" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="N30" t="s">
+        <v>72</v>
+      </c>
+      <c r="O30">
+        <v>1100</v>
       </c>
       <c r="P30">
-        <v>1100</v>
+        <v>2000</v>
       </c>
       <c r="Q30">
-        <v>2000</v>
-      </c>
-      <c r="R30">
         <v>14.40793180682512</v>
       </c>
     </row>
-    <row r="31" spans="1:18">
+    <row r="31" spans="1:17">
       <c r="A31" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B31">
         <v>48.88259682475478</v>
@@ -2311,27 +2218,24 @@
         <v>4.67</v>
       </c>
       <c r="M31" t="s">
-        <v>71</v>
-      </c>
-      <c r="N31">
-        <v>18</v>
-      </c>
-      <c r="O31" t="s">
-        <v>73</v>
+        <v>70</v>
+      </c>
+      <c r="N31" t="s">
+        <v>72</v>
+      </c>
+      <c r="O31">
+        <v>1200</v>
       </c>
       <c r="P31">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="Q31">
-        <v>2000</v>
-      </c>
-      <c r="R31">
         <v>14.10148343125805</v>
       </c>
     </row>
-    <row r="32" spans="1:18">
+    <row r="32" spans="1:17">
       <c r="A32" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B32">
         <v>50.17</v>
@@ -2367,27 +2271,24 @@
         <v>4.95</v>
       </c>
       <c r="M32" t="s">
-        <v>67</v>
-      </c>
-      <c r="N32">
-        <v>22</v>
-      </c>
-      <c r="O32" t="s">
-        <v>73</v>
+        <v>66</v>
+      </c>
+      <c r="N32" t="s">
+        <v>72</v>
+      </c>
+      <c r="O32">
+        <v>1250</v>
       </c>
       <c r="P32">
-        <v>1250</v>
+        <v>2000</v>
       </c>
       <c r="Q32">
-        <v>2000</v>
-      </c>
-      <c r="R32">
         <v>14.84090081974931</v>
       </c>
     </row>
-    <row r="33" spans="1:18">
+    <row r="33" spans="1:17">
       <c r="A33" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B33">
         <v>49.64</v>
@@ -2423,27 +2324,24 @@
         <v>4.8</v>
       </c>
       <c r="M33" t="s">
-        <v>68</v>
-      </c>
-      <c r="N33">
-        <v>5</v>
-      </c>
-      <c r="O33" t="s">
-        <v>73</v>
+        <v>67</v>
+      </c>
+      <c r="N33" t="s">
+        <v>72</v>
+      </c>
+      <c r="O33">
+        <v>1200</v>
       </c>
       <c r="P33">
-        <v>1200</v>
+        <v>2021</v>
       </c>
       <c r="Q33">
-        <v>2021</v>
-      </c>
-      <c r="R33">
         <v>14.12735099987323</v>
       </c>
     </row>
-    <row r="34" spans="1:18">
+    <row r="34" spans="1:17">
       <c r="A34" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B34">
         <v>49.64</v>
@@ -2479,27 +2377,24 @@
         <v>4.46</v>
       </c>
       <c r="M34" t="s">
-        <v>69</v>
-      </c>
-      <c r="N34">
-        <v>5</v>
-      </c>
-      <c r="O34" t="s">
-        <v>73</v>
+        <v>68</v>
+      </c>
+      <c r="N34" t="s">
+        <v>72</v>
+      </c>
+      <c r="O34">
+        <v>1200</v>
       </c>
       <c r="P34">
-        <v>1200</v>
+        <v>2033</v>
       </c>
       <c r="Q34">
-        <v>2033</v>
-      </c>
-      <c r="R34">
         <v>13.25934825976636</v>
       </c>
     </row>
-    <row r="35" spans="1:18">
+    <row r="35" spans="1:17">
       <c r="A35" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B35">
         <v>49.4</v>
@@ -2535,27 +2430,24 @@
         <v>4.92</v>
       </c>
       <c r="M35" t="s">
-        <v>64</v>
-      </c>
-      <c r="N35">
-        <v>6</v>
-      </c>
-      <c r="O35" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N35" t="s">
+        <v>72</v>
+      </c>
+      <c r="O35">
+        <v>1200</v>
       </c>
       <c r="P35">
-        <v>1200</v>
+        <v>2059</v>
       </c>
       <c r="Q35">
-        <v>2059</v>
-      </c>
-      <c r="R35">
         <v>14.72313029408801</v>
       </c>
     </row>
-    <row r="36" spans="1:18">
+    <row r="36" spans="1:17">
       <c r="A36" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B36">
         <v>49.4</v>
@@ -2591,27 +2483,24 @@
         <v>5.19</v>
       </c>
       <c r="M36" t="s">
-        <v>64</v>
-      </c>
-      <c r="N36">
-        <v>6</v>
-      </c>
-      <c r="O36" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N36" t="s">
+        <v>72</v>
+      </c>
+      <c r="O36">
+        <v>1200</v>
       </c>
       <c r="P36">
-        <v>1200</v>
+        <v>2138</v>
       </c>
       <c r="Q36">
-        <v>2138</v>
-      </c>
-      <c r="R36">
         <v>15.40662502191551</v>
       </c>
     </row>
-    <row r="37" spans="1:18">
+    <row r="37" spans="1:17">
       <c r="A37" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B37">
         <v>49.4</v>
@@ -2647,27 +2536,24 @@
         <v>5.99</v>
       </c>
       <c r="M37" t="s">
-        <v>64</v>
-      </c>
-      <c r="N37">
-        <v>6</v>
-      </c>
-      <c r="O37" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N37" t="s">
+        <v>72</v>
+      </c>
+      <c r="O37">
+        <v>1200</v>
       </c>
       <c r="P37">
-        <v>1200</v>
+        <v>2760</v>
       </c>
       <c r="Q37">
-        <v>2760</v>
-      </c>
-      <c r="R37">
         <v>17.36896095070735</v>
       </c>
     </row>
-    <row r="38" spans="1:18">
+    <row r="38" spans="1:17">
       <c r="A38" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B38">
         <v>50.71</v>
@@ -2703,27 +2589,24 @@
         <v>5.93</v>
       </c>
       <c r="M38" t="s">
-        <v>70</v>
-      </c>
-      <c r="N38">
-        <v>2</v>
-      </c>
-      <c r="O38" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="N38" t="s">
+        <v>72</v>
+      </c>
+      <c r="O38">
+        <v>1100</v>
       </c>
       <c r="P38">
-        <v>1100</v>
+        <v>3000</v>
       </c>
       <c r="Q38">
-        <v>3000</v>
-      </c>
-      <c r="R38">
         <v>17.86281654945389</v>
       </c>
     </row>
-    <row r="39" spans="1:18">
+    <row r="39" spans="1:17">
       <c r="A39" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B39">
         <v>50.17</v>
@@ -2759,27 +2642,24 @@
         <v>6.25</v>
       </c>
       <c r="M39" t="s">
-        <v>67</v>
-      </c>
-      <c r="N39">
-        <v>22</v>
-      </c>
-      <c r="O39" t="s">
-        <v>73</v>
+        <v>66</v>
+      </c>
+      <c r="N39" t="s">
+        <v>72</v>
+      </c>
+      <c r="O39">
+        <v>1250</v>
       </c>
       <c r="P39">
-        <v>1250</v>
+        <v>3000</v>
       </c>
       <c r="Q39">
-        <v>3000</v>
-      </c>
-      <c r="R39">
         <v>18.03555546561759</v>
       </c>
     </row>
-    <row r="40" spans="1:18">
+    <row r="40" spans="1:17">
       <c r="A40" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B40">
         <v>49.64</v>
@@ -2815,27 +2695,24 @@
         <v>6.27</v>
       </c>
       <c r="M40" t="s">
-        <v>68</v>
-      </c>
-      <c r="N40">
-        <v>5</v>
-      </c>
-      <c r="O40" t="s">
-        <v>73</v>
+        <v>67</v>
+      </c>
+      <c r="N40" t="s">
+        <v>72</v>
+      </c>
+      <c r="O40">
+        <v>1200</v>
       </c>
       <c r="P40">
-        <v>1200</v>
+        <v>3043</v>
       </c>
       <c r="Q40">
-        <v>3043</v>
-      </c>
-      <c r="R40">
         <v>17.68855662136642</v>
       </c>
     </row>
-    <row r="41" spans="1:18">
+    <row r="41" spans="1:17">
       <c r="A41" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B41">
         <v>49.4</v>
@@ -2871,27 +2748,24 @@
         <v>7.74</v>
       </c>
       <c r="M41" t="s">
-        <v>64</v>
-      </c>
-      <c r="N41">
-        <v>6</v>
-      </c>
-      <c r="O41" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="N41" t="s">
+        <v>72</v>
+      </c>
+      <c r="O41">
+        <v>1200</v>
       </c>
       <c r="P41">
-        <v>1200</v>
+        <v>3842</v>
       </c>
       <c r="Q41">
-        <v>3842</v>
-      </c>
-      <c r="R41">
         <v>21.35949795573888</v>
       </c>
     </row>
-    <row r="42" spans="1:18">
+    <row r="42" spans="1:17">
       <c r="A42" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B42">
         <v>50.71</v>
@@ -2927,27 +2801,24 @@
         <v>7.3</v>
       </c>
       <c r="M42" t="s">
-        <v>70</v>
-      </c>
-      <c r="N42">
-        <v>2</v>
-      </c>
-      <c r="O42" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="N42" t="s">
+        <v>72</v>
+      </c>
+      <c r="O42">
+        <v>1100</v>
       </c>
       <c r="P42">
-        <v>1100</v>
+        <v>4000</v>
       </c>
       <c r="Q42">
-        <v>4000</v>
-      </c>
-      <c r="R42">
         <v>21.11813141655405</v>
       </c>
     </row>
-    <row r="43" spans="1:18">
+    <row r="43" spans="1:17">
       <c r="A43" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43">
         <v>48.45657568238214</v>
@@ -2983,27 +2854,24 @@
         <v>7.57</v>
       </c>
       <c r="M43" t="s">
-        <v>72</v>
-      </c>
-      <c r="N43">
-        <v>9</v>
-      </c>
-      <c r="O43" t="s">
-        <v>73</v>
+        <v>71</v>
+      </c>
+      <c r="N43" t="s">
+        <v>72</v>
+      </c>
+      <c r="O43">
+        <v>1200</v>
       </c>
       <c r="P43">
-        <v>1200</v>
+        <v>5000</v>
       </c>
       <c r="Q43">
-        <v>5000</v>
-      </c>
-      <c r="R43">
         <v>20.69448942240509</v>
       </c>
     </row>
-    <row r="44" spans="1:18">
+    <row r="44" spans="1:17">
       <c r="A44" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B44">
         <v>50.17</v>
@@ -3039,27 +2907,24 @@
         <v>8.81</v>
       </c>
       <c r="M44" t="s">
-        <v>67</v>
-      </c>
-      <c r="N44">
-        <v>22</v>
-      </c>
-      <c r="O44" t="s">
-        <v>73</v>
+        <v>66</v>
+      </c>
+      <c r="N44" t="s">
+        <v>72</v>
+      </c>
+      <c r="O44">
+        <v>1250</v>
       </c>
       <c r="P44">
-        <v>1250</v>
+        <v>5000</v>
       </c>
       <c r="Q44">
-        <v>5000</v>
-      </c>
-      <c r="R44">
         <v>23.67403216850881</v>
       </c>
     </row>
-    <row r="45" spans="1:18">
+    <row r="45" spans="1:17">
       <c r="A45" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B45">
         <v>49.64</v>
@@ -3095,27 +2960,24 @@
         <v>9.380000000000001</v>
       </c>
       <c r="M45" t="s">
-        <v>69</v>
-      </c>
-      <c r="N45">
-        <v>5</v>
-      </c>
-      <c r="O45" t="s">
-        <v>73</v>
+        <v>68</v>
+      </c>
+      <c r="N45" t="s">
+        <v>72</v>
+      </c>
+      <c r="O45">
+        <v>1200</v>
       </c>
       <c r="P45">
-        <v>1200</v>
+        <v>5009</v>
       </c>
       <c r="Q45">
-        <v>5009</v>
-      </c>
-      <c r="R45">
         <v>24.32784238062053</v>
       </c>
     </row>
-    <row r="46" spans="1:18">
+    <row r="46" spans="1:17">
       <c r="A46" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B46">
         <v>49.64</v>
@@ -3151,27 +3013,24 @@
         <v>9.380000000000001</v>
       </c>
       <c r="M46" t="s">
-        <v>68</v>
-      </c>
-      <c r="N46">
-        <v>5</v>
-      </c>
-      <c r="O46" t="s">
-        <v>73</v>
+        <v>67</v>
+      </c>
+      <c r="N46" t="s">
+        <v>72</v>
+      </c>
+      <c r="O46">
+        <v>1200</v>
       </c>
       <c r="P46">
-        <v>1200</v>
+        <v>5009</v>
       </c>
       <c r="Q46">
-        <v>5009</v>
-      </c>
-      <c r="R46">
         <v>24.32784238062053</v>
       </c>
     </row>
-    <row r="47" spans="1:18">
+    <row r="47" spans="1:17">
       <c r="A47" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B47">
         <v>50.71</v>
@@ -3207,27 +3066,24 @@
         <v>8.51</v>
       </c>
       <c r="M47" t="s">
-        <v>70</v>
-      </c>
-      <c r="N47">
-        <v>2</v>
-      </c>
-      <c r="O47" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="N47" t="s">
+        <v>72</v>
+      </c>
+      <c r="O47">
+        <v>1100</v>
       </c>
       <c r="P47">
-        <v>1100</v>
+        <v>5343</v>
       </c>
       <c r="Q47">
-        <v>5343</v>
-      </c>
-      <c r="R47">
         <v>23.78593068400964</v>
       </c>
     </row>
-    <row r="48" spans="1:18">
+    <row r="48" spans="1:17">
       <c r="A48" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B48">
         <v>50.71</v>
@@ -3263,21 +3119,18 @@
         <v>9.369999999999999</v>
       </c>
       <c r="M48" t="s">
-        <v>70</v>
-      </c>
-      <c r="N48">
-        <v>2</v>
-      </c>
-      <c r="O48" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="N48" t="s">
+        <v>72</v>
+      </c>
+      <c r="O48">
+        <v>1100</v>
       </c>
       <c r="P48">
-        <v>1100</v>
+        <v>6067</v>
       </c>
       <c r="Q48">
-        <v>6067</v>
-      </c>
-      <c r="R48">
         <v>25.57492242692672</v>
       </c>
     </row>

</xml_diff>